<commit_message>
dependences implementation when deleting one thing, big work
</commit_message>
<xml_diff>
--- a/portfolio-simulator/data/data_profil.xlsx
+++ b/portfolio-simulator/data/data_profil.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5160" yWindow="2475" windowWidth="21600" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="930" yWindow="2700" windowWidth="21600" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Metiers" sheetId="1" state="visible" r:id="rId1"/>
@@ -428,11 +428,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
-  <cols>
-    <col width="19.85546875" bestFit="1" customWidth="1" min="9" max="9"/>
-  </cols>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -457,40 +454,35 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>ID SALAIRE</t>
+          <t>DATE IN</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>DATE IN</t>
+          <t>DATE OUT</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>DATE OUT</t>
+          <t>INTITULE</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>INTITULE</t>
+          <t>ANNUEL BRUT (€/AN)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>ANNUEL BRUT (€/AN)</t>
+          <t>ANNUEL NET (€/AN)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>ANNUEL NET (€/AN)</t>
+          <t>PAS (%)</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
-        <is>
-          <t>PAS (%)</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
         <is>
           <t>PRIVE</t>
         </is>
@@ -514,30 +506,27 @@
       <c r="D3" t="n">
         <v>3000000001</v>
       </c>
-      <c r="E3" t="n">
-        <v>9000000005</v>
-      </c>
-      <c r="F3" s="1" t="n">
+      <c r="E3" s="3" t="n">
         <v>45901</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="F3" s="3" t="n">
         <v>46143</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Acadomia</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>3600</v>
+      </c>
       <c r="I3" t="n">
-        <v>3600</v>
+        <v>3000</v>
       </c>
       <c r="J3" t="n">
-        <v>3000</v>
-      </c>
-      <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
@@ -556,30 +545,27 @@
       <c r="D4" t="n">
         <v>3000000004</v>
       </c>
-      <c r="E4" t="n">
-        <v>9000000009</v>
-      </c>
-      <c r="F4" s="1" t="n">
+      <c r="E4" s="3" t="n">
         <v>46143</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="F4" s="3" t="n">
         <v>62214</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>riche</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>2500000</v>
+      </c>
       <c r="I4" t="n">
-        <v>2500000</v>
+        <v>250000</v>
       </c>
       <c r="J4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="K4" t="n">
         <v>15</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
@@ -598,30 +584,27 @@
       <c r="D5" t="n">
         <v>3000000005</v>
       </c>
-      <c r="E5" t="n">
-        <v>9000000011</v>
-      </c>
-      <c r="F5" s="1" t="n">
+      <c r="E5" s="3" t="n">
         <v>46204</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="F5" s="3" t="n">
         <v>49857</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Pompier</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>18000</v>
+      </c>
       <c r="I5" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="J5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
@@ -640,32 +623,68 @@
       <c r="D6" t="n">
         <v>3000000005</v>
       </c>
-      <c r="E6" t="n">
-        <v>9000000012</v>
-      </c>
-      <c r="F6" s="1" t="n">
+      <c r="E6" s="3" t="n">
         <v>46204</v>
       </c>
-      <c r="G6" s="1" t="n">
+      <c r="F6" s="3" t="n">
         <v>50222</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Professeur de Sport</t>
         </is>
       </c>
+      <c r="H6" t="n">
+        <v>18000</v>
+      </c>
       <c r="I6" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="J6" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K6" t="n">
         <v>5</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5000000005</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>45839</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>58654</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ingénieur</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>40000</v>
+      </c>
+      <c r="J7" t="n">
+        <v>10</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -680,10 +699,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="10.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="11.7109375" bestFit="1" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -766,13 +784,51 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>reprise test</t>
+          <t>Test reprise</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="E5" s="1" t="n">
+        <v>109911</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6000000004</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ajout error.py</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>109911</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Test dependances</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E7" s="1" t="n">
         <v>109911</v>
       </c>
     </row>
@@ -1038,7 +1094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1069,55 +1125,45 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>ID DEPENSE</t>
+          <t>ID SOURCE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>ID RECETTE</t>
+          <t>DATE IN</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>ID INVEST</t>
+          <t>DATE OUT</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>DATE IN</t>
+          <t>MONTANT</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>DATE OUT</t>
+          <t>DUREE DIFF (MOIS)</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>MONTANT</t>
+          <t>DUREE (MOIS)</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>DUREE DIFF (MOIS)</t>
+          <t>MENSUALITE (€)</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>DUREE (MOIS)</t>
+          <t>TAUX (%)</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
-        <is>
-          <t>MENSUALITE (€)</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>TAUX (%)</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
         <is>
           <t>TYPE</t>
         </is>
@@ -1144,28 +1190,28 @@
       <c r="E3" t="n">
         <v>1000000000</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="G3" s="3" t="n">
         <v>44197</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="H3" s="3" t="n">
         <v>49157</v>
       </c>
+      <c r="I3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J3" t="n">
+        <v>60</v>
+      </c>
       <c r="K3" t="n">
-        <v>10000</v>
+        <v>103</v>
       </c>
       <c r="L3" t="n">
-        <v>60</v>
+        <v>128</v>
       </c>
       <c r="M3" t="n">
-        <v>103</v>
-      </c>
-      <c r="N3" t="n">
-        <v>128</v>
-      </c>
-      <c r="O3" t="n">
         <v>3</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Mensualité Constante</t>
         </is>
@@ -1188,36 +1234,30 @@
         <v>1000000000</v>
       </c>
       <c r="F4" t="n">
-        <v>8000000004</v>
-      </c>
-      <c r="G4" t="n">
-        <v>9000000013</v>
-      </c>
-      <c r="H4" t="n">
         <v>7000000002</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="G4" s="3" t="n">
         <v>47543</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="H4" s="3" t="n">
         <v>58166</v>
       </c>
+      <c r="I4" t="n">
+        <v>225000</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
       <c r="K4" t="n">
-        <v>225000</v>
+        <v>349</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>850</v>
       </c>
       <c r="M4" t="n">
-        <v>349</v>
-      </c>
-      <c r="N4" t="n">
-        <v>850</v>
-      </c>
-      <c r="O4" t="n">
         <v>2</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Mensualité Constante</t>
         </is>
@@ -1240,36 +1280,30 @@
         <v>1000000000</v>
       </c>
       <c r="F5" t="n">
-        <v>8000000007</v>
-      </c>
-      <c r="G5" t="n">
-        <v>9000000018</v>
-      </c>
-      <c r="H5" t="n">
         <v>7000000003</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="G5" s="3" t="n">
         <v>46813</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="H5" s="3" t="n">
         <v>56250</v>
       </c>
+      <c r="I5" t="n">
+        <v>108000</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
       <c r="K5" t="n">
-        <v>108000</v>
+        <v>310</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="M5" t="n">
-        <v>310</v>
-      </c>
-      <c r="N5" t="n">
-        <v>500</v>
-      </c>
-      <c r="O5" t="n">
         <v>3</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Mensualité Constante</t>
         </is>
@@ -1292,36 +1326,122 @@
         <v>1000000000</v>
       </c>
       <c r="F6" t="n">
-        <v>8000000009</v>
-      </c>
-      <c r="G6" t="n">
-        <v>9000000022</v>
-      </c>
-      <c r="H6" t="n">
         <v>7000000004</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="G6" s="3" t="n">
         <v>47178</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="H6" s="3" t="n">
         <v>48549</v>
       </c>
+      <c r="I6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
       <c r="K6" t="n">
-        <v>9000</v>
+        <v>45</v>
       </c>
       <c r="L6" t="n">
+        <v>200</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Mensualité Constante</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4000000005</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2000000002</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>7000000007</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>54424</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="M6" t="n">
-        <v>45</v>
-      </c>
-      <c r="N6" t="n">
-        <v>200</v>
-      </c>
-      <c r="O6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="K7" t="n">
+        <v>243</v>
+      </c>
+      <c r="L7" t="n">
+        <v>50</v>
+      </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Mensualité Constante</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4000000006</v>
+      </c>
+      <c r="B8" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2000000002</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7000000008</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>52628</v>
+      </c>
+      <c r="I8" t="n">
+        <v>108000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>153</v>
+      </c>
+      <c r="L8" t="n">
+        <v>800</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>Mensualité Constante</t>
         </is>
@@ -1412,13 +1532,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
-  <cols>
-    <col width="4.7109375" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="5.140625" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="19.140625" bestFit="1" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1634,6 +1749,31 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="B8" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2000000002</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Courant</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1648,7 +1788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1679,7 +1819,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>ID INVEST</t>
+          <t>ID SOURCE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -2025,6 +2165,249 @@
         <v>10000</v>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>Ponctuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8000000011</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6000000003</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3000000005</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>46508</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>48427</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>hj</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Loyers</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>600</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8000000012</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7000000007</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>54424</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>crédit 243 mois 10 000,00 €</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Crédit</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>50</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8000000013</v>
+      </c>
+      <c r="C13" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7000000007</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Achat Dulong</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Investissement</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>90000</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Ponctuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>8000000016</v>
+      </c>
+      <c r="C14" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>47362</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>47362</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Voiture</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Autres</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>100000</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Ponctuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>8000000017</v>
+      </c>
+      <c r="C15" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4000000006</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>52628</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>crédit 153 mois 108 000,00 €</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Crédit</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>800</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>8000000018</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7000000008</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Achat asas</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Investissement</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>120000</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>Ponctuel</t>
         </is>
@@ -2041,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2072,7 +2455,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>ID INVEST</t>
+          <t>ID SOURCE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -2837,7 +3220,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>9000000024</v>
+        <v>9000000026</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
@@ -2853,68 +3236,64 @@
         <v>7000000004</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>47604</v>
+        <v>48245</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>48245</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ipi</t>
+          <t>Vente ipi</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Locataires</t>
+          <t>Investissement</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>1000</v>
+        <v>10303.00999999997</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Mensuel</t>
-        </is>
-      </c>
-      <c r="M20" t="n">
-        <v>0.01</v>
-      </c>
+          <t>Ponctuel</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>9000000026</v>
+        <v>9000000027</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>6000000003</v>
+        <v>6000000005</v>
       </c>
       <c r="D21" t="n">
         <v>1000000000</v>
       </c>
       <c r="E21" t="n">
-        <v>3000000005</v>
-      </c>
-      <c r="F21" t="n">
-        <v>7000000004</v>
-      </c>
+        <v>3000000006</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" s="3" t="n">
-        <v>48245</v>
+        <v>46235</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>48245</v>
+        <v>46235</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Vente ipi</t>
+          <t>Ouverture compte</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Investissement</t>
+          <t>Dépots</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>10303.00999999997</v>
+        <v>0</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -2922,6 +3301,266 @@
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>9000000028</v>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5000000005</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>45839</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>58654</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Ingénieur</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Revenus</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>9000000029</v>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7000000007</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>crédit 243 mois 10 000,00 €</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Crédit</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>10000</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Ponctuel</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>9000000030</v>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7000000007</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>49583</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Dulong</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Locataires</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>9000000032</v>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" s="3" t="n">
+        <v>47331</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>47331</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Loto</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Dons/Cadeaux</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>100000</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Ponctuel</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9000000033</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4000000006</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>crédit 153 mois 108 000,00 €</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Crédit</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>108000</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Ponctuel</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>9000000034</v>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="F27" t="n">
+        <v>7000000008</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>51257</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>asas</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Locataires</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>500</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>0.02</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2934,7 +3573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2965,62 +3604,57 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>PRIX ACHAT</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>TITRE</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>LOCALISATION</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>SURFACE</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>TYPE</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>COMPTANT (%)</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>VALORISATION (%/AN)</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>DATE ACHAT</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>DATE VENTE</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ETAT</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>ID ACHAT</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>ID VENTE</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>PRIX ACHAT</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>TITRE</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>LOCALISATION</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>SURFACE</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>TYPE</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>COMPTANT (%)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>VALORISATION (%/AN)</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>DATE ACHAT</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>DATE VENTE</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>ETAT</t>
         </is>
       </c>
     </row>
@@ -3037,26 +3671,23 @@
         <v>4000000000</v>
       </c>
       <c r="F2" t="n">
-        <v>8000000000</v>
-      </c>
-      <c r="H2" t="n">
         <v>100000</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>pars</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="K2" t="n">
         <v>0.1</v>
       </c>
-      <c r="N2" t="n">
+      <c r="L2" t="n">
         <v>0.06</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="M2" s="3" t="n">
         <v>47239</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>47239</v>
       </c>
     </row>
@@ -3077,45 +3708,39 @@
         <v>4000000002</v>
       </c>
       <c r="F3" t="n">
-        <v>8000000005</v>
-      </c>
-      <c r="G3" t="n">
-        <v>9000000015</v>
-      </c>
-      <c r="H3" t="n">
         <v>250000</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Achat RS</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>50</v>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>50</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
         <v>0.1</v>
       </c>
-      <c r="N3" t="n">
+      <c r="L3" t="n">
         <v>0.025</v>
       </c>
-      <c r="O3" s="3" t="n">
+      <c r="M3" s="3" t="n">
         <v>47543</v>
       </c>
-      <c r="P3" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>49735</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>vendu</t>
         </is>
@@ -3138,45 +3763,39 @@
         <v>4000000003</v>
       </c>
       <c r="F4" t="n">
-        <v>8000000008</v>
-      </c>
-      <c r="G4" t="n">
-        <v>9000000019</v>
-      </c>
-      <c r="H4" t="n">
         <v>120000</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>caca</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>100</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
         <v>0.1</v>
       </c>
-      <c r="N4" t="n">
+      <c r="L4" t="n">
         <v>0.03</v>
       </c>
-      <c r="O4" s="3" t="n">
+      <c r="M4" s="3" t="n">
         <v>46813</v>
       </c>
-      <c r="P4" s="3" t="n">
+      <c r="N4" s="3" t="n">
         <v>54970</v>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>vendu</t>
         </is>
@@ -3199,48 +3818,253 @@
         <v>4000000004</v>
       </c>
       <c r="F5" t="n">
-        <v>8000000010</v>
-      </c>
-      <c r="G5" t="n">
-        <v>9000000026</v>
-      </c>
-      <c r="H5" t="n">
         <v>10000</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>ipi</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>50</v>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>T1 BIS</t>
         </is>
       </c>
       <c r="K5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>47178</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>48245</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>vendu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>7000000005</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6000000004</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4000000005</v>
+      </c>
+      <c r="F6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>pipi</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>mtp</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>50</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>47635</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>48792</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>vendu</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7000000006</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6000000003</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3000000005</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>oui p</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>120</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>T1 BIS</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="K7" t="n">
         <v>0.1</v>
       </c>
-      <c r="N5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>47178</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>48245</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>vendu</t>
-        </is>
+      <c r="L7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>48000</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>à créditer</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7000000007</v>
+      </c>
+      <c r="B8" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4000000005</v>
+      </c>
+      <c r="F8" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Dulong</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Studio</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>47027</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>actif</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7000000008</v>
+      </c>
+      <c r="B9" t="n">
+        <v>6000000005</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3000000006</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4000000006</v>
+      </c>
+      <c r="F9" t="n">
+        <v>120000</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>asas</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>as</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>15</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>T1 BIS</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>47969</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>actif</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>8000000018</v>
       </c>
     </row>
   </sheetData>
@@ -3256,6 +4080,11 @@
   </sheetPr>
   <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="15.140625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="21.5703125" bestFit="1" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>